<commit_message>
Adapter la grille Excel au site (décisions post-réunion médecins)
Site conservé tel quel (décisions validées) :
- Terminologie : PM (pas MR)
- Synthèse & Lisibilité : critère unique fusionné (MR)
- Impression globale : critère MR final, hors bloc Correspondance
- Correspondance profil → CR : PM
- 7 blocs avec les noms du site

Excel mis à jour en conséquence :
- Grille : Terminologie → PM, col Synthèse & Lisibilité (fusion S&L + Lisibilité), Impression globale ajoutée
- Guidelines : réorganisation critères 16-20 + bloc "6. Cohérence & Impression"

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/grille_evaluation_CR.xlsx
+++ b/grille_evaluation_CR.xlsx
@@ -281,7 +281,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -441,6 +441,24 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1060,7 +1078,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1871,27 +1889,27 @@
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">  5. Forme</t>
+          <t xml:space="preserve">  5. Rédaction</t>
         </is>
       </c>
     </row>
     <row r="24" ht="65" customHeight="1">
-      <c r="A24" s="26" t="inlineStr">
+      <c r="A24" s="18" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
-      <c r="B24" s="27" t="inlineStr">
+      <c r="B24" s="19" t="inlineStr">
         <is>
           <t>Terminologie</t>
         </is>
       </c>
-      <c r="C24" s="26" t="inlineStr">
-        <is>
-          <t>MR</t>
-        </is>
-      </c>
-      <c r="D24" s="28" t="inlineStr">
+      <c r="C24" s="18" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="D24" s="20" t="inlineStr">
         <is>
           <t>Vérifier que le vocabulaire radiothérapeutique est correct et standardisé en français : termes de fractionnement, dosimétrie, volumes (GTV, CTV, PTV), techniques.</t>
         </is>
@@ -1930,7 +1948,7 @@
       </c>
       <c r="B25" s="27" t="inlineStr">
         <is>
-          <t>Lisibilité &amp; style</t>
+          <t>Organisation</t>
         </is>
       </c>
       <c r="C25" s="26" t="inlineStr">
@@ -1940,7 +1958,7 @@
       </c>
       <c r="D25" s="28" t="inlineStr">
         <is>
-          <t>Évaluer si le texte est fluide, naturel et adapté au style d'un compte rendu médical français : ton professionnel, phrases bien construites, absence de répétitions maladroites.</t>
+          <t>Évaluer si le CR suit une structure logique et claire : contexte clinique → diagnostic → traitement → tolérance → bilan → suivi. Les informations doivent être dans un ordre cohérent.</t>
         </is>
       </c>
       <c r="E25" s="21" t="inlineStr">
@@ -1977,7 +1995,7 @@
       </c>
       <c r="B26" s="27" t="inlineStr">
         <is>
-          <t>Organisation</t>
+          <t>Synthèse &amp; Lisibilité</t>
         </is>
       </c>
       <c r="C26" s="26" t="inlineStr">
@@ -1987,137 +2005,131 @@
       </c>
       <c r="D26" s="28" t="inlineStr">
         <is>
-          <t>Évaluer si le CR suit une structure logique et claire : contexte clinique → diagnostic → traitement → tolérance → bilan → suivi. Les informations doivent être dans un ordre cohérent.</t>
+          <t>Évaluer si le texte est fluide, naturel et adapté au style d'un CR médical, et si le CR est concis et va à l'essentiel : absence de répétitions, style professionnel, lisibilité générale.</t>
         </is>
       </c>
       <c r="E26" s="21" t="inlineStr">
         <is>
-          <t>Structure absente ou chaotique, informations mélangées sans logique.</t>
+          <t>Texte illisible ou clairement non médical, avec répétitions majeures.</t>
         </is>
       </c>
       <c r="F26" s="22" t="inlineStr">
         <is>
-          <t>Structure partielle, plusieurs sections dans le désordre.</t>
+          <t>Texte compréhensible mais avec des maladresses stylistiques ou répétitions notables.</t>
         </is>
       </c>
       <c r="G26" s="23" t="inlineStr">
         <is>
-          <t>Structure globalement logique avec quelques éléments mal positionnés.</t>
+          <t>Texte globalement fluide avec quelques légères imperfections de style ou concision.</t>
         </is>
       </c>
       <c r="H26" s="24" t="inlineStr">
         <is>
-          <t>Structure claire et logique respectant l'ordre attendu d'un CR de radiothérapie.</t>
-        </is>
-      </c>
-      <c r="I26" s="25" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+          <t>Texte naturel, fluide, parfaitement adapté au style d'un CR médical, concis et sans répétition.</t>
+        </is>
+      </c>
+      <c r="I26" s="25" t="n"/>
     </row>
     <row r="27" ht="65" customHeight="1">
-      <c r="A27" s="26" t="inlineStr">
+      <c r="A27" s="18" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="B27" s="27" t="inlineStr">
-        <is>
-          <t>Synthèse</t>
-        </is>
-      </c>
-      <c r="C27" s="26" t="inlineStr">
-        <is>
-          <t>MR</t>
-        </is>
-      </c>
-      <c r="D27" s="28" t="inlineStr">
-        <is>
-          <t>Évaluer si le CR est concis et va à l'essentiel : absence de répétitions inutiles, d'informations non pertinentes ou de longueurs excessives.</t>
+      <c r="B27" s="19" t="inlineStr">
+        <is>
+          <t>Correspondance profil → CR</t>
+        </is>
+      </c>
+      <c r="C27" s="18" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="D27" s="20" t="inlineStr">
+        <is>
+          <t>⚠ Nécessite le profil patient (seed) sous les yeux. Vérifier que les informations clés du CR (stade, chirurgie, ER/PR, chimiothérapie, âge…) correspondent au profil patient fourni comme données d'entrée.
+⚠ Note : le profil peut être reformulé (pas repris mot pour mot) dans le CR — cela est considéré comme correct.</t>
         </is>
       </c>
       <c r="E27" s="21" t="inlineStr">
         <is>
-          <t>CR très verbeux avec de nombreuses répétitions ou informations hors sujet.</t>
+          <t>Le CR contient des informations qui contredisent directement le profil patient (stade différent, chirurgie incorrecte…).</t>
         </is>
       </c>
       <c r="F27" s="22" t="inlineStr">
         <is>
-          <t>Quelques répétitions ou longueurs notables affectant la lisibilité.</t>
+          <t>Plusieurs informations du CR ne correspondent pas au profil patient.</t>
         </is>
       </c>
       <c r="G27" s="23" t="inlineStr">
         <is>
-          <t>CR globalement concis avec quelques redondances mineures.</t>
+          <t>Le CR correspond globalement au profil patient avec une légère divergence mineure.</t>
         </is>
       </c>
       <c r="H27" s="24" t="inlineStr">
         <is>
-          <t>CR parfaitement concis, pertinent, sans répétition ni information superflue.</t>
+          <t>Le CR reflète fidèlement toutes les informations clés du profil patient.</t>
         </is>
       </c>
       <c r="I27" s="25" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Profil patient non disponible pour cette évaluation.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">  6. Correspondance profil → CR</t>
+          <t xml:space="preserve">  6. Cohérence &amp; Impression</t>
         </is>
       </c>
     </row>
     <row r="29" ht="65" customHeight="1">
-      <c r="A29" s="18" t="inlineStr">
+      <c r="A29" s="26" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="B29" s="19" t="inlineStr">
-        <is>
-          <t>Correspondance profil → CR</t>
-        </is>
-      </c>
-      <c r="C29" s="18" t="inlineStr">
-        <is>
-          <t>PM</t>
-        </is>
-      </c>
-      <c r="D29" s="20" t="inlineStr">
-        <is>
-          <t>⚠ Nécessite le profil patient (seed) sous les yeux. Vérifier que les informations clés du CR (stade, chirurgie, ER/PR, chimiothérapie, âge…) correspondent au profil patient fourni comme données d'entrée.
-⚠ Note : le profil peut être reformulé (pas repris mot pour mot) dans le CR — cela est considéré comme correct.</t>
+      <c r="B29" s="27" t="inlineStr">
+        <is>
+          <t>Impression globale</t>
+        </is>
+      </c>
+      <c r="C29" s="26" t="inlineStr">
+        <is>
+          <t>MR</t>
+        </is>
+      </c>
+      <c r="D29" s="28" t="inlineStr">
+        <is>
+          <t>Quelle est votre impression globale ? Ce CR est-il acceptable pour une utilisation clinique réelle ? Prendre en compte l'ensemble des critères évalués.</t>
         </is>
       </c>
       <c r="E29" s="21" t="inlineStr">
         <is>
-          <t>Le CR contient des informations qui contredisent directement le profil patient (stade différent, chirurgie incorrecte…).</t>
+          <t>CR inacceptable : erreurs majeures.</t>
         </is>
       </c>
       <c r="F29" s="22" t="inlineStr">
         <is>
-          <t>Plusieurs informations du CR ne correspondent pas au profil patient.</t>
+          <t>CR nécessitant des corrections importantes.</t>
         </is>
       </c>
       <c r="G29" s="23" t="inlineStr">
         <is>
-          <t>Le CR correspond globalement au profil patient avec une légère divergence mineure.</t>
+          <t>CR globalement acceptable avec quelques réserves.</t>
         </is>
       </c>
       <c r="H29" s="24" t="inlineStr">
         <is>
-          <t>Le CR reflète fidèlement toutes les informations clés du profil patient.</t>
-        </is>
-      </c>
-      <c r="I29" s="25" t="inlineStr">
-        <is>
-          <t>Profil patient non disponible pour cette évaluation.</t>
-        </is>
-      </c>
-    </row>
+          <t>CR parfaitement acceptable et prêt pour une utilisation clinique.</t>
+        </is>
+      </c>
+      <c r="I29" s="25" t="n"/>
+    </row>
+    <row r="30"/>
+    <row r="31"/>
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="A2:I2"/>
@@ -2257,18 +2269,19 @@
         </is>
       </c>
       <c r="V4" s="34" t="n"/>
-      <c r="W4" s="36" t="inlineStr">
-        <is>
-          <t>5. Forme</t>
-        </is>
-      </c>
+      <c r="W4" s="35" t="inlineStr">
+        <is>
+          <t>5. Rédaction</t>
+        </is>
+      </c>
+      <c r="Z4" s="34" t="n"/>
       <c r="AA4" s="34" t="n"/>
       <c r="AB4" s="35" t="inlineStr">
         <is>
-          <t>6. Correspondance profil → CR</t>
-        </is>
-      </c>
-      <c r="AC4" s="34" t="n"/>
+          <t>6. Cohérence &amp; Impression</t>
+        </is>
+      </c>
+      <c r="AC4" s="57" t="n"/>
       <c r="AD4" s="38" t="inlineStr">
         <is>
           <t>Commentaires
@@ -2365,33 +2378,33 @@
         </is>
       </c>
       <c r="V5" s="34" t="n"/>
-      <c r="W5" s="42" t="inlineStr">
+      <c r="W5" s="41" t="inlineStr">
+        <is>
+          <t>Physicien Médical</t>
+        </is>
+      </c>
+      <c r="X5" s="42" t="inlineStr">
         <is>
           <t>Médecin Radiothérapeute</t>
         </is>
       </c>
-      <c r="X5" s="42" t="inlineStr">
+      <c r="Y5" s="42" t="inlineStr">
         <is>
           <t>Médecin Radiothérapeute</t>
         </is>
       </c>
-      <c r="Y5" s="42" t="inlineStr">
-        <is>
-          <t>Médecin Radiothérapeute</t>
-        </is>
-      </c>
-      <c r="Z5" s="42" t="inlineStr">
-        <is>
-          <t>Médecin Radiothérapeute</t>
-        </is>
-      </c>
+      <c r="Z5" s="58" t="n"/>
       <c r="AA5" s="34" t="n"/>
       <c r="AB5" s="41" t="inlineStr">
         <is>
           <t>Physicien Médical</t>
         </is>
       </c>
-      <c r="AC5" s="34" t="n"/>
+      <c r="AC5" s="57" t="inlineStr">
+        <is>
+          <t>Médecin Radiothérapeute</t>
+        </is>
+      </c>
       <c r="AD5" s="40" t="n"/>
       <c r="AE5" s="40" t="n"/>
     </row>
@@ -2478,33 +2491,33 @@
         </is>
       </c>
       <c r="V6" s="34" t="n"/>
-      <c r="W6" s="44" t="inlineStr">
+      <c r="W6" s="43" t="inlineStr">
         <is>
           <t>Terminologie</t>
         </is>
       </c>
       <c r="X6" s="44" t="inlineStr">
         <is>
-          <t>Lisibilité &amp; style</t>
+          <t>Organisation</t>
         </is>
       </c>
       <c r="Y6" s="44" t="inlineStr">
         <is>
-          <t>Organisation</t>
-        </is>
-      </c>
-      <c r="Z6" s="44" t="inlineStr">
-        <is>
-          <t>Synthèse</t>
-        </is>
-      </c>
+          <t>Synthèse &amp; Lisibilité</t>
+        </is>
+      </c>
+      <c r="Z6" s="59" t="n"/>
       <c r="AA6" s="34" t="n"/>
       <c r="AB6" s="43" t="inlineStr">
         <is>
           <t>Correspondance profil → CR</t>
         </is>
       </c>
-      <c r="AC6" s="34" t="n"/>
+      <c r="AC6" s="60" t="inlineStr">
+        <is>
+          <t>Impression globale</t>
+        </is>
+      </c>
       <c r="AD6" s="40" t="n"/>
       <c r="AE6" s="40" t="n"/>
     </row>
@@ -2598,7 +2611,7 @@
         </is>
       </c>
       <c r="V7" s="34" t="n"/>
-      <c r="W7" s="46" t="inlineStr">
+      <c r="W7" s="45" t="inlineStr">
         <is>
           <t>Le vocabulaire radiothérapeutique français est-il correct et standard ?
 (fractionnement, dosimétrie, champs tangentiels…)</t>
@@ -2606,20 +2619,17 @@
       </c>
       <c r="X7" s="46" t="inlineStr">
         <is>
-          <t>Le texte est-il naturel et fluide ? Le style rédactionnel est-il adapté à un compte rendu médical ?</t>
-        </is>
-      </c>
-      <c r="Y7" s="46" t="inlineStr">
-        <is>
           <t>Le CR suit-il une structure logique et claire ? Les informations sont-elles présentées dans un ordre cohérent ?
 (contexte → diagnostic → traitement → suivi)</t>
         </is>
       </c>
-      <c r="Z7" s="46" t="inlineStr">
-        <is>
-          <t>Le CR est-il concis et pertinent ? Évite-t-il les répétitions inutiles et les informations redondantes ?</t>
-        </is>
-      </c>
+      <c r="Y7" s="46" t="inlineStr">
+        <is>
+          <t>Le texte est-il fluide, concis et adapté au style médical ?
+(lisibilité, concision, absence de répétitions)</t>
+        </is>
+      </c>
+      <c r="Z7" s="61" t="n"/>
       <c r="AA7" s="34" t="n"/>
       <c r="AB7" s="45" t="inlineStr">
         <is>
@@ -2628,7 +2638,12 @@
 ⚠ Note : le profil peut être reformulé (pas repris mot pour mot) dans le CR — cela est considéré comme correct.</t>
         </is>
       </c>
-      <c r="AC7" s="34" t="n"/>
+      <c r="AC7" s="62" t="inlineStr">
+        <is>
+          <t>Quelle est votre impression globale ?
+Ce CR est-il acceptable pour une utilisation clinique ?</t>
+        </is>
+      </c>
       <c r="AD7" s="40" t="n"/>
       <c r="AE7" s="40" t="n"/>
     </row>
@@ -2715,7 +2730,7 @@
         </is>
       </c>
       <c r="V8" s="34" t="n"/>
-      <c r="W8" s="49" t="inlineStr">
+      <c r="W8" s="48" t="inlineStr">
         <is>
           <t>1 · 2 · 3 · 4</t>
         </is>
@@ -2730,18 +2745,18 @@
           <t>1 · 2 · 3 · 4</t>
         </is>
       </c>
-      <c r="Z8" s="49" t="inlineStr">
-        <is>
-          <t>1 · 2 · 3 · 4</t>
-        </is>
-      </c>
+      <c r="Z8" s="63" t="n"/>
       <c r="AA8" s="34" t="n"/>
       <c r="AB8" s="48" t="inlineStr">
         <is>
           <t>1 · 2 · 3 · 4 · N/A</t>
         </is>
       </c>
-      <c r="AC8" s="34" t="n"/>
+      <c r="AC8" s="60" t="inlineStr">
+        <is>
+          <t>1 · 2 · 3 · 4</t>
+        </is>
+      </c>
       <c r="AD8" s="47" t="n"/>
       <c r="AE8" s="47" t="n"/>
     </row>
@@ -2776,13 +2791,13 @@
       <c r="T9" s="53" t="inlineStr"/>
       <c r="U9" s="53" t="inlineStr"/>
       <c r="V9" s="34" t="n"/>
-      <c r="W9" s="53" t="inlineStr"/>
-      <c r="X9" s="53" t="inlineStr"/>
-      <c r="Y9" s="53" t="inlineStr"/>
-      <c r="Z9" s="53" t="inlineStr"/>
+      <c r="W9" s="52" t="inlineStr"/>
+      <c r="X9" s="53" t="n"/>
+      <c r="Y9" s="53" t="n"/>
+      <c r="Z9" s="64" t="n"/>
       <c r="AA9" s="34" t="n"/>
       <c r="AB9" s="52" t="inlineStr"/>
-      <c r="AC9" s="34" t="n"/>
+      <c r="AC9" s="62" t="n"/>
       <c r="AD9" s="54" t="inlineStr"/>
       <c r="AE9" s="55" t="inlineStr"/>
     </row>
@@ -2817,13 +2832,13 @@
       <c r="T10" s="53" t="inlineStr"/>
       <c r="U10" s="53" t="inlineStr"/>
       <c r="V10" s="34" t="n"/>
-      <c r="W10" s="53" t="inlineStr"/>
-      <c r="X10" s="53" t="inlineStr"/>
-      <c r="Y10" s="53" t="inlineStr"/>
-      <c r="Z10" s="53" t="inlineStr"/>
+      <c r="W10" s="52" t="inlineStr"/>
+      <c r="X10" s="53" t="n"/>
+      <c r="Y10" s="53" t="n"/>
+      <c r="Z10" s="64" t="n"/>
       <c r="AA10" s="34" t="n"/>
       <c r="AB10" s="52" t="inlineStr"/>
-      <c r="AC10" s="34" t="n"/>
+      <c r="AC10" s="62" t="n"/>
       <c r="AD10" s="54" t="inlineStr"/>
       <c r="AE10" s="55" t="inlineStr"/>
     </row>
@@ -2858,13 +2873,13 @@
       <c r="T11" s="53" t="inlineStr"/>
       <c r="U11" s="53" t="inlineStr"/>
       <c r="V11" s="34" t="n"/>
-      <c r="W11" s="53" t="inlineStr"/>
-      <c r="X11" s="53" t="inlineStr"/>
-      <c r="Y11" s="53" t="inlineStr"/>
-      <c r="Z11" s="53" t="inlineStr"/>
+      <c r="W11" s="52" t="inlineStr"/>
+      <c r="X11" s="53" t="n"/>
+      <c r="Y11" s="53" t="n"/>
+      <c r="Z11" s="64" t="n"/>
       <c r="AA11" s="34" t="n"/>
       <c r="AB11" s="52" t="inlineStr"/>
-      <c r="AC11" s="34" t="n"/>
+      <c r="AC11" s="62" t="n"/>
       <c r="AD11" s="54" t="inlineStr"/>
       <c r="AE11" s="55" t="inlineStr"/>
     </row>
@@ -2899,13 +2914,13 @@
       <c r="T12" s="53" t="inlineStr"/>
       <c r="U12" s="53" t="inlineStr"/>
       <c r="V12" s="34" t="n"/>
-      <c r="W12" s="53" t="inlineStr"/>
-      <c r="X12" s="53" t="inlineStr"/>
-      <c r="Y12" s="53" t="inlineStr"/>
-      <c r="Z12" s="53" t="inlineStr"/>
+      <c r="W12" s="52" t="inlineStr"/>
+      <c r="X12" s="53" t="n"/>
+      <c r="Y12" s="53" t="n"/>
+      <c r="Z12" s="64" t="n"/>
       <c r="AA12" s="34" t="n"/>
       <c r="AB12" s="52" t="inlineStr"/>
-      <c r="AC12" s="34" t="n"/>
+      <c r="AC12" s="62" t="n"/>
       <c r="AD12" s="54" t="inlineStr"/>
       <c r="AE12" s="55" t="inlineStr"/>
     </row>
@@ -2940,13 +2955,13 @@
       <c r="T13" s="53" t="inlineStr"/>
       <c r="U13" s="53" t="inlineStr"/>
       <c r="V13" s="34" t="n"/>
-      <c r="W13" s="53" t="inlineStr"/>
-      <c r="X13" s="53" t="inlineStr"/>
-      <c r="Y13" s="53" t="inlineStr"/>
-      <c r="Z13" s="53" t="inlineStr"/>
+      <c r="W13" s="52" t="inlineStr"/>
+      <c r="X13" s="53" t="n"/>
+      <c r="Y13" s="53" t="n"/>
+      <c r="Z13" s="64" t="n"/>
       <c r="AA13" s="34" t="n"/>
       <c r="AB13" s="52" t="inlineStr"/>
-      <c r="AC13" s="34" t="n"/>
+      <c r="AC13" s="62" t="n"/>
       <c r="AD13" s="54" t="inlineStr"/>
       <c r="AE13" s="55" t="inlineStr"/>
     </row>
@@ -2981,13 +2996,13 @@
       <c r="T14" s="53" t="inlineStr"/>
       <c r="U14" s="53" t="inlineStr"/>
       <c r="V14" s="34" t="n"/>
-      <c r="W14" s="53" t="inlineStr"/>
-      <c r="X14" s="53" t="inlineStr"/>
-      <c r="Y14" s="53" t="inlineStr"/>
-      <c r="Z14" s="53" t="inlineStr"/>
+      <c r="W14" s="52" t="inlineStr"/>
+      <c r="X14" s="53" t="n"/>
+      <c r="Y14" s="53" t="n"/>
+      <c r="Z14" s="64" t="n"/>
       <c r="AA14" s="34" t="n"/>
       <c r="AB14" s="52" t="inlineStr"/>
-      <c r="AC14" s="34" t="n"/>
+      <c r="AC14" s="62" t="n"/>
       <c r="AD14" s="54" t="inlineStr"/>
       <c r="AE14" s="55" t="inlineStr"/>
     </row>
@@ -3022,13 +3037,13 @@
       <c r="T15" s="53" t="inlineStr"/>
       <c r="U15" s="53" t="inlineStr"/>
       <c r="V15" s="34" t="n"/>
-      <c r="W15" s="53" t="inlineStr"/>
-      <c r="X15" s="53" t="inlineStr"/>
-      <c r="Y15" s="53" t="inlineStr"/>
-      <c r="Z15" s="53" t="inlineStr"/>
+      <c r="W15" s="52" t="inlineStr"/>
+      <c r="X15" s="53" t="n"/>
+      <c r="Y15" s="53" t="n"/>
+      <c r="Z15" s="64" t="n"/>
       <c r="AA15" s="34" t="n"/>
       <c r="AB15" s="52" t="inlineStr"/>
-      <c r="AC15" s="34" t="n"/>
+      <c r="AC15" s="62" t="n"/>
       <c r="AD15" s="54" t="inlineStr"/>
       <c r="AE15" s="55" t="inlineStr"/>
     </row>
@@ -3063,13 +3078,13 @@
       <c r="T16" s="53" t="inlineStr"/>
       <c r="U16" s="53" t="inlineStr"/>
       <c r="V16" s="34" t="n"/>
-      <c r="W16" s="53" t="inlineStr"/>
-      <c r="X16" s="53" t="inlineStr"/>
-      <c r="Y16" s="53" t="inlineStr"/>
-      <c r="Z16" s="53" t="inlineStr"/>
+      <c r="W16" s="52" t="inlineStr"/>
+      <c r="X16" s="53" t="n"/>
+      <c r="Y16" s="53" t="n"/>
+      <c r="Z16" s="64" t="n"/>
       <c r="AA16" s="34" t="n"/>
       <c r="AB16" s="52" t="inlineStr"/>
-      <c r="AC16" s="34" t="n"/>
+      <c r="AC16" s="62" t="n"/>
       <c r="AD16" s="54" t="inlineStr"/>
       <c r="AE16" s="55" t="inlineStr"/>
     </row>
@@ -3104,13 +3119,13 @@
       <c r="T17" s="53" t="inlineStr"/>
       <c r="U17" s="53" t="inlineStr"/>
       <c r="V17" s="34" t="n"/>
-      <c r="W17" s="53" t="inlineStr"/>
-      <c r="X17" s="53" t="inlineStr"/>
-      <c r="Y17" s="53" t="inlineStr"/>
-      <c r="Z17" s="53" t="inlineStr"/>
+      <c r="W17" s="52" t="inlineStr"/>
+      <c r="X17" s="53" t="n"/>
+      <c r="Y17" s="53" t="n"/>
+      <c r="Z17" s="64" t="n"/>
       <c r="AA17" s="34" t="n"/>
       <c r="AB17" s="52" t="inlineStr"/>
-      <c r="AC17" s="34" t="n"/>
+      <c r="AC17" s="62" t="n"/>
       <c r="AD17" s="54" t="inlineStr"/>
       <c r="AE17" s="55" t="inlineStr"/>
     </row>
@@ -3145,13 +3160,13 @@
       <c r="T18" s="53" t="inlineStr"/>
       <c r="U18" s="53" t="inlineStr"/>
       <c r="V18" s="34" t="n"/>
-      <c r="W18" s="53" t="inlineStr"/>
-      <c r="X18" s="53" t="inlineStr"/>
-      <c r="Y18" s="53" t="inlineStr"/>
-      <c r="Z18" s="53" t="inlineStr"/>
+      <c r="W18" s="52" t="inlineStr"/>
+      <c r="X18" s="53" t="n"/>
+      <c r="Y18" s="53" t="n"/>
+      <c r="Z18" s="64" t="n"/>
       <c r="AA18" s="34" t="n"/>
       <c r="AB18" s="52" t="inlineStr"/>
-      <c r="AC18" s="34" t="n"/>
+      <c r="AC18" s="62" t="n"/>
       <c r="AD18" s="54" t="inlineStr"/>
       <c r="AE18" s="55" t="inlineStr"/>
     </row>
@@ -3186,13 +3201,13 @@
       <c r="T19" s="53" t="inlineStr"/>
       <c r="U19" s="53" t="inlineStr"/>
       <c r="V19" s="34" t="n"/>
-      <c r="W19" s="53" t="inlineStr"/>
-      <c r="X19" s="53" t="inlineStr"/>
-      <c r="Y19" s="53" t="inlineStr"/>
-      <c r="Z19" s="53" t="inlineStr"/>
+      <c r="W19" s="52" t="inlineStr"/>
+      <c r="X19" s="53" t="n"/>
+      <c r="Y19" s="53" t="n"/>
+      <c r="Z19" s="64" t="n"/>
       <c r="AA19" s="34" t="n"/>
       <c r="AB19" s="52" t="inlineStr"/>
-      <c r="AC19" s="34" t="n"/>
+      <c r="AC19" s="62" t="n"/>
       <c r="AD19" s="54" t="inlineStr"/>
       <c r="AE19" s="55" t="inlineStr"/>
     </row>
@@ -3227,13 +3242,13 @@
       <c r="T20" s="53" t="inlineStr"/>
       <c r="U20" s="53" t="inlineStr"/>
       <c r="V20" s="34" t="n"/>
-      <c r="W20" s="53" t="inlineStr"/>
-      <c r="X20" s="53" t="inlineStr"/>
-      <c r="Y20" s="53" t="inlineStr"/>
-      <c r="Z20" s="53" t="inlineStr"/>
+      <c r="W20" s="52" t="inlineStr"/>
+      <c r="X20" s="53" t="n"/>
+      <c r="Y20" s="53" t="n"/>
+      <c r="Z20" s="64" t="n"/>
       <c r="AA20" s="34" t="n"/>
       <c r="AB20" s="52" t="inlineStr"/>
-      <c r="AC20" s="34" t="n"/>
+      <c r="AC20" s="62" t="n"/>
       <c r="AD20" s="54" t="inlineStr"/>
       <c r="AE20" s="55" t="inlineStr"/>
     </row>
@@ -3268,13 +3283,13 @@
       <c r="T21" s="53" t="inlineStr"/>
       <c r="U21" s="53" t="inlineStr"/>
       <c r="V21" s="34" t="n"/>
-      <c r="W21" s="53" t="inlineStr"/>
-      <c r="X21" s="53" t="inlineStr"/>
-      <c r="Y21" s="53" t="inlineStr"/>
-      <c r="Z21" s="53" t="inlineStr"/>
+      <c r="W21" s="52" t="inlineStr"/>
+      <c r="X21" s="53" t="n"/>
+      <c r="Y21" s="53" t="n"/>
+      <c r="Z21" s="64" t="n"/>
       <c r="AA21" s="34" t="n"/>
       <c r="AB21" s="52" t="inlineStr"/>
-      <c r="AC21" s="34" t="n"/>
+      <c r="AC21" s="62" t="n"/>
       <c r="AD21" s="54" t="inlineStr"/>
       <c r="AE21" s="55" t="inlineStr"/>
     </row>
@@ -3309,13 +3324,13 @@
       <c r="T22" s="53" t="inlineStr"/>
       <c r="U22" s="53" t="inlineStr"/>
       <c r="V22" s="34" t="n"/>
-      <c r="W22" s="53" t="inlineStr"/>
-      <c r="X22" s="53" t="inlineStr"/>
-      <c r="Y22" s="53" t="inlineStr"/>
-      <c r="Z22" s="53" t="inlineStr"/>
+      <c r="W22" s="52" t="inlineStr"/>
+      <c r="X22" s="53" t="n"/>
+      <c r="Y22" s="53" t="n"/>
+      <c r="Z22" s="64" t="n"/>
       <c r="AA22" s="34" t="n"/>
       <c r="AB22" s="52" t="inlineStr"/>
-      <c r="AC22" s="34" t="n"/>
+      <c r="AC22" s="62" t="n"/>
       <c r="AD22" s="54" t="inlineStr"/>
       <c r="AE22" s="55" t="inlineStr"/>
     </row>
@@ -3350,13 +3365,13 @@
       <c r="T23" s="53" t="inlineStr"/>
       <c r="U23" s="53" t="inlineStr"/>
       <c r="V23" s="34" t="n"/>
-      <c r="W23" s="53" t="inlineStr"/>
-      <c r="X23" s="53" t="inlineStr"/>
-      <c r="Y23" s="53" t="inlineStr"/>
-      <c r="Z23" s="53" t="inlineStr"/>
+      <c r="W23" s="52" t="inlineStr"/>
+      <c r="X23" s="53" t="n"/>
+      <c r="Y23" s="53" t="n"/>
+      <c r="Z23" s="64" t="n"/>
       <c r="AA23" s="34" t="n"/>
       <c r="AB23" s="52" t="inlineStr"/>
-      <c r="AC23" s="34" t="n"/>
+      <c r="AC23" s="62" t="n"/>
       <c r="AD23" s="54" t="inlineStr"/>
       <c r="AE23" s="55" t="inlineStr"/>
     </row>
@@ -3391,13 +3406,13 @@
       <c r="T24" s="53" t="inlineStr"/>
       <c r="U24" s="53" t="inlineStr"/>
       <c r="V24" s="34" t="n"/>
-      <c r="W24" s="53" t="inlineStr"/>
-      <c r="X24" s="53" t="inlineStr"/>
-      <c r="Y24" s="53" t="inlineStr"/>
-      <c r="Z24" s="53" t="inlineStr"/>
+      <c r="W24" s="52" t="inlineStr"/>
+      <c r="X24" s="53" t="n"/>
+      <c r="Y24" s="53" t="n"/>
+      <c r="Z24" s="64" t="n"/>
       <c r="AA24" s="34" t="n"/>
       <c r="AB24" s="52" t="inlineStr"/>
-      <c r="AC24" s="34" t="n"/>
+      <c r="AC24" s="62" t="n"/>
       <c r="AD24" s="54" t="inlineStr"/>
       <c r="AE24" s="55" t="inlineStr"/>
     </row>
@@ -3432,13 +3447,13 @@
       <c r="T25" s="53" t="inlineStr"/>
       <c r="U25" s="53" t="inlineStr"/>
       <c r="V25" s="34" t="n"/>
-      <c r="W25" s="53" t="inlineStr"/>
-      <c r="X25" s="53" t="inlineStr"/>
-      <c r="Y25" s="53" t="inlineStr"/>
-      <c r="Z25" s="53" t="inlineStr"/>
+      <c r="W25" s="52" t="inlineStr"/>
+      <c r="X25" s="53" t="n"/>
+      <c r="Y25" s="53" t="n"/>
+      <c r="Z25" s="64" t="n"/>
       <c r="AA25" s="34" t="n"/>
       <c r="AB25" s="52" t="inlineStr"/>
-      <c r="AC25" s="34" t="n"/>
+      <c r="AC25" s="62" t="n"/>
       <c r="AD25" s="54" t="inlineStr"/>
       <c r="AE25" s="55" t="inlineStr"/>
     </row>
@@ -3473,13 +3488,13 @@
       <c r="T26" s="53" t="inlineStr"/>
       <c r="U26" s="53" t="inlineStr"/>
       <c r="V26" s="34" t="n"/>
-      <c r="W26" s="53" t="inlineStr"/>
-      <c r="X26" s="53" t="inlineStr"/>
-      <c r="Y26" s="53" t="inlineStr"/>
-      <c r="Z26" s="53" t="inlineStr"/>
+      <c r="W26" s="52" t="inlineStr"/>
+      <c r="X26" s="53" t="n"/>
+      <c r="Y26" s="53" t="n"/>
+      <c r="Z26" s="64" t="n"/>
       <c r="AA26" s="34" t="n"/>
       <c r="AB26" s="52" t="inlineStr"/>
-      <c r="AC26" s="34" t="n"/>
+      <c r="AC26" s="62" t="n"/>
       <c r="AD26" s="54" t="inlineStr"/>
       <c r="AE26" s="55" t="inlineStr"/>
     </row>
@@ -3514,13 +3529,13 @@
       <c r="T27" s="53" t="inlineStr"/>
       <c r="U27" s="53" t="inlineStr"/>
       <c r="V27" s="34" t="n"/>
-      <c r="W27" s="53" t="inlineStr"/>
-      <c r="X27" s="53" t="inlineStr"/>
-      <c r="Y27" s="53" t="inlineStr"/>
-      <c r="Z27" s="53" t="inlineStr"/>
+      <c r="W27" s="52" t="inlineStr"/>
+      <c r="X27" s="53" t="n"/>
+      <c r="Y27" s="53" t="n"/>
+      <c r="Z27" s="64" t="n"/>
       <c r="AA27" s="34" t="n"/>
       <c r="AB27" s="52" t="inlineStr"/>
-      <c r="AC27" s="34" t="n"/>
+      <c r="AC27" s="62" t="n"/>
       <c r="AD27" s="54" t="inlineStr"/>
       <c r="AE27" s="55" t="inlineStr"/>
     </row>
@@ -3555,13 +3570,13 @@
       <c r="T28" s="53" t="inlineStr"/>
       <c r="U28" s="53" t="inlineStr"/>
       <c r="V28" s="34" t="n"/>
-      <c r="W28" s="53" t="inlineStr"/>
-      <c r="X28" s="53" t="inlineStr"/>
-      <c r="Y28" s="53" t="inlineStr"/>
-      <c r="Z28" s="53" t="inlineStr"/>
+      <c r="W28" s="52" t="inlineStr"/>
+      <c r="X28" s="53" t="n"/>
+      <c r="Y28" s="53" t="n"/>
+      <c r="Z28" s="64" t="n"/>
       <c r="AA28" s="34" t="n"/>
       <c r="AB28" s="52" t="inlineStr"/>
-      <c r="AC28" s="34" t="n"/>
+      <c r="AC28" s="62" t="n"/>
       <c r="AD28" s="54" t="inlineStr"/>
       <c r="AE28" s="55" t="inlineStr"/>
     </row>
@@ -3596,13 +3611,13 @@
       <c r="T29" s="53" t="inlineStr"/>
       <c r="U29" s="53" t="inlineStr"/>
       <c r="V29" s="34" t="n"/>
-      <c r="W29" s="53" t="inlineStr"/>
-      <c r="X29" s="53" t="inlineStr"/>
-      <c r="Y29" s="53" t="inlineStr"/>
-      <c r="Z29" s="53" t="inlineStr"/>
+      <c r="W29" s="52" t="inlineStr"/>
+      <c r="X29" s="53" t="n"/>
+      <c r="Y29" s="53" t="n"/>
+      <c r="Z29" s="64" t="n"/>
       <c r="AA29" s="34" t="n"/>
       <c r="AB29" s="52" t="inlineStr"/>
-      <c r="AC29" s="34" t="n"/>
+      <c r="AC29" s="62" t="n"/>
       <c r="AD29" s="54" t="inlineStr"/>
       <c r="AE29" s="55" t="inlineStr"/>
     </row>
@@ -3637,13 +3652,13 @@
       <c r="T30" s="53" t="inlineStr"/>
       <c r="U30" s="53" t="inlineStr"/>
       <c r="V30" s="34" t="n"/>
-      <c r="W30" s="53" t="inlineStr"/>
-      <c r="X30" s="53" t="inlineStr"/>
-      <c r="Y30" s="53" t="inlineStr"/>
-      <c r="Z30" s="53" t="inlineStr"/>
+      <c r="W30" s="52" t="inlineStr"/>
+      <c r="X30" s="53" t="n"/>
+      <c r="Y30" s="53" t="n"/>
+      <c r="Z30" s="64" t="n"/>
       <c r="AA30" s="34" t="n"/>
       <c r="AB30" s="52" t="inlineStr"/>
-      <c r="AC30" s="34" t="n"/>
+      <c r="AC30" s="62" t="n"/>
       <c r="AD30" s="54" t="inlineStr"/>
       <c r="AE30" s="55" t="inlineStr"/>
     </row>
@@ -3678,13 +3693,13 @@
       <c r="T31" s="53" t="inlineStr"/>
       <c r="U31" s="53" t="inlineStr"/>
       <c r="V31" s="34" t="n"/>
-      <c r="W31" s="53" t="inlineStr"/>
-      <c r="X31" s="53" t="inlineStr"/>
-      <c r="Y31" s="53" t="inlineStr"/>
-      <c r="Z31" s="53" t="inlineStr"/>
+      <c r="W31" s="52" t="inlineStr"/>
+      <c r="X31" s="53" t="n"/>
+      <c r="Y31" s="53" t="n"/>
+      <c r="Z31" s="64" t="n"/>
       <c r="AA31" s="34" t="n"/>
       <c r="AB31" s="52" t="inlineStr"/>
-      <c r="AC31" s="34" t="n"/>
+      <c r="AC31" s="62" t="n"/>
       <c r="AD31" s="54" t="inlineStr"/>
       <c r="AE31" s="55" t="inlineStr"/>
     </row>
@@ -3719,13 +3734,13 @@
       <c r="T32" s="53" t="inlineStr"/>
       <c r="U32" s="53" t="inlineStr"/>
       <c r="V32" s="34" t="n"/>
-      <c r="W32" s="53" t="inlineStr"/>
-      <c r="X32" s="53" t="inlineStr"/>
-      <c r="Y32" s="53" t="inlineStr"/>
-      <c r="Z32" s="53" t="inlineStr"/>
+      <c r="W32" s="52" t="inlineStr"/>
+      <c r="X32" s="53" t="n"/>
+      <c r="Y32" s="53" t="n"/>
+      <c r="Z32" s="64" t="n"/>
       <c r="AA32" s="34" t="n"/>
       <c r="AB32" s="52" t="inlineStr"/>
-      <c r="AC32" s="34" t="n"/>
+      <c r="AC32" s="62" t="n"/>
       <c r="AD32" s="54" t="inlineStr"/>
       <c r="AE32" s="55" t="inlineStr"/>
     </row>
@@ -3760,13 +3775,13 @@
       <c r="T33" s="53" t="inlineStr"/>
       <c r="U33" s="53" t="inlineStr"/>
       <c r="V33" s="34" t="n"/>
-      <c r="W33" s="53" t="inlineStr"/>
-      <c r="X33" s="53" t="inlineStr"/>
-      <c r="Y33" s="53" t="inlineStr"/>
-      <c r="Z33" s="53" t="inlineStr"/>
+      <c r="W33" s="52" t="inlineStr"/>
+      <c r="X33" s="53" t="n"/>
+      <c r="Y33" s="53" t="n"/>
+      <c r="Z33" s="64" t="n"/>
       <c r="AA33" s="34" t="n"/>
       <c r="AB33" s="52" t="inlineStr"/>
-      <c r="AC33" s="34" t="n"/>
+      <c r="AC33" s="62" t="n"/>
       <c r="AD33" s="54" t="inlineStr"/>
       <c r="AE33" s="55" t="inlineStr"/>
     </row>
@@ -3801,13 +3816,13 @@
       <c r="T34" s="53" t="inlineStr"/>
       <c r="U34" s="53" t="inlineStr"/>
       <c r="V34" s="34" t="n"/>
-      <c r="W34" s="53" t="inlineStr"/>
-      <c r="X34" s="53" t="inlineStr"/>
-      <c r="Y34" s="53" t="inlineStr"/>
-      <c r="Z34" s="53" t="inlineStr"/>
+      <c r="W34" s="52" t="inlineStr"/>
+      <c r="X34" s="53" t="n"/>
+      <c r="Y34" s="53" t="n"/>
+      <c r="Z34" s="64" t="n"/>
       <c r="AA34" s="34" t="n"/>
       <c r="AB34" s="52" t="inlineStr"/>
-      <c r="AC34" s="34" t="n"/>
+      <c r="AC34" s="62" t="n"/>
       <c r="AD34" s="54" t="inlineStr"/>
       <c r="AE34" s="55" t="inlineStr"/>
     </row>
@@ -3842,13 +3857,13 @@
       <c r="T35" s="53" t="inlineStr"/>
       <c r="U35" s="53" t="inlineStr"/>
       <c r="V35" s="34" t="n"/>
-      <c r="W35" s="53" t="inlineStr"/>
-      <c r="X35" s="53" t="inlineStr"/>
-      <c r="Y35" s="53" t="inlineStr"/>
-      <c r="Z35" s="53" t="inlineStr"/>
+      <c r="W35" s="52" t="inlineStr"/>
+      <c r="X35" s="53" t="n"/>
+      <c r="Y35" s="53" t="n"/>
+      <c r="Z35" s="64" t="n"/>
       <c r="AA35" s="34" t="n"/>
       <c r="AB35" s="52" t="inlineStr"/>
-      <c r="AC35" s="34" t="n"/>
+      <c r="AC35" s="62" t="n"/>
       <c r="AD35" s="54" t="inlineStr"/>
       <c r="AE35" s="55" t="inlineStr"/>
     </row>
@@ -3883,13 +3898,13 @@
       <c r="T36" s="53" t="inlineStr"/>
       <c r="U36" s="53" t="inlineStr"/>
       <c r="V36" s="34" t="n"/>
-      <c r="W36" s="53" t="inlineStr"/>
-      <c r="X36" s="53" t="inlineStr"/>
-      <c r="Y36" s="53" t="inlineStr"/>
-      <c r="Z36" s="53" t="inlineStr"/>
+      <c r="W36" s="52" t="inlineStr"/>
+      <c r="X36" s="53" t="n"/>
+      <c r="Y36" s="53" t="n"/>
+      <c r="Z36" s="64" t="n"/>
       <c r="AA36" s="34" t="n"/>
       <c r="AB36" s="52" t="inlineStr"/>
-      <c r="AC36" s="34" t="n"/>
+      <c r="AC36" s="62" t="n"/>
       <c r="AD36" s="54" t="inlineStr"/>
       <c r="AE36" s="55" t="inlineStr"/>
     </row>
@@ -3924,13 +3939,13 @@
       <c r="T37" s="53" t="inlineStr"/>
       <c r="U37" s="53" t="inlineStr"/>
       <c r="V37" s="34" t="n"/>
-      <c r="W37" s="53" t="inlineStr"/>
-      <c r="X37" s="53" t="inlineStr"/>
-      <c r="Y37" s="53" t="inlineStr"/>
-      <c r="Z37" s="53" t="inlineStr"/>
+      <c r="W37" s="52" t="inlineStr"/>
+      <c r="X37" s="53" t="n"/>
+      <c r="Y37" s="53" t="n"/>
+      <c r="Z37" s="64" t="n"/>
       <c r="AA37" s="34" t="n"/>
       <c r="AB37" s="52" t="inlineStr"/>
-      <c r="AC37" s="34" t="n"/>
+      <c r="AC37" s="62" t="n"/>
       <c r="AD37" s="54" t="inlineStr"/>
       <c r="AE37" s="55" t="inlineStr"/>
     </row>
@@ -3965,13 +3980,13 @@
       <c r="T38" s="53" t="inlineStr"/>
       <c r="U38" s="53" t="inlineStr"/>
       <c r="V38" s="34" t="n"/>
-      <c r="W38" s="53" t="inlineStr"/>
-      <c r="X38" s="53" t="inlineStr"/>
-      <c r="Y38" s="53" t="inlineStr"/>
-      <c r="Z38" s="53" t="inlineStr"/>
+      <c r="W38" s="52" t="inlineStr"/>
+      <c r="X38" s="53" t="n"/>
+      <c r="Y38" s="53" t="n"/>
+      <c r="Z38" s="64" t="n"/>
       <c r="AA38" s="34" t="n"/>
       <c r="AB38" s="52" t="inlineStr"/>
-      <c r="AC38" s="34" t="n"/>
+      <c r="AC38" s="62" t="n"/>
       <c r="AD38" s="54" t="inlineStr"/>
       <c r="AE38" s="55" t="inlineStr"/>
     </row>
@@ -4006,13 +4021,13 @@
       <c r="T39" s="53" t="inlineStr"/>
       <c r="U39" s="53" t="inlineStr"/>
       <c r="V39" s="34" t="n"/>
-      <c r="W39" s="53" t="inlineStr"/>
-      <c r="X39" s="53" t="inlineStr"/>
-      <c r="Y39" s="53" t="inlineStr"/>
-      <c r="Z39" s="53" t="inlineStr"/>
+      <c r="W39" s="52" t="inlineStr"/>
+      <c r="X39" s="53" t="n"/>
+      <c r="Y39" s="53" t="n"/>
+      <c r="Z39" s="64" t="n"/>
       <c r="AA39" s="34" t="n"/>
       <c r="AB39" s="52" t="inlineStr"/>
-      <c r="AC39" s="34" t="n"/>
+      <c r="AC39" s="62" t="n"/>
       <c r="AD39" s="54" t="inlineStr"/>
       <c r="AE39" s="55" t="inlineStr"/>
     </row>
@@ -4047,13 +4062,13 @@
       <c r="T40" s="53" t="inlineStr"/>
       <c r="U40" s="53" t="inlineStr"/>
       <c r="V40" s="34" t="n"/>
-      <c r="W40" s="53" t="inlineStr"/>
-      <c r="X40" s="53" t="inlineStr"/>
-      <c r="Y40" s="53" t="inlineStr"/>
-      <c r="Z40" s="53" t="inlineStr"/>
+      <c r="W40" s="52" t="inlineStr"/>
+      <c r="X40" s="53" t="n"/>
+      <c r="Y40" s="53" t="n"/>
+      <c r="Z40" s="64" t="n"/>
       <c r="AA40" s="34" t="n"/>
       <c r="AB40" s="52" t="inlineStr"/>
-      <c r="AC40" s="34" t="n"/>
+      <c r="AC40" s="62" t="n"/>
       <c r="AD40" s="54" t="inlineStr"/>
       <c r="AE40" s="55" t="inlineStr"/>
     </row>
@@ -4088,13 +4103,13 @@
       <c r="T41" s="53" t="inlineStr"/>
       <c r="U41" s="53" t="inlineStr"/>
       <c r="V41" s="34" t="n"/>
-      <c r="W41" s="53" t="inlineStr"/>
-      <c r="X41" s="53" t="inlineStr"/>
-      <c r="Y41" s="53" t="inlineStr"/>
-      <c r="Z41" s="53" t="inlineStr"/>
+      <c r="W41" s="52" t="inlineStr"/>
+      <c r="X41" s="53" t="n"/>
+      <c r="Y41" s="53" t="n"/>
+      <c r="Z41" s="64" t="n"/>
       <c r="AA41" s="34" t="n"/>
       <c r="AB41" s="52" t="inlineStr"/>
-      <c r="AC41" s="34" t="n"/>
+      <c r="AC41" s="62" t="n"/>
       <c r="AD41" s="54" t="inlineStr"/>
       <c r="AE41" s="55" t="inlineStr"/>
     </row>
@@ -4129,13 +4144,13 @@
       <c r="T42" s="53" t="inlineStr"/>
       <c r="U42" s="53" t="inlineStr"/>
       <c r="V42" s="34" t="n"/>
-      <c r="W42" s="53" t="inlineStr"/>
-      <c r="X42" s="53" t="inlineStr"/>
-      <c r="Y42" s="53" t="inlineStr"/>
-      <c r="Z42" s="53" t="inlineStr"/>
+      <c r="W42" s="52" t="inlineStr"/>
+      <c r="X42" s="53" t="n"/>
+      <c r="Y42" s="53" t="n"/>
+      <c r="Z42" s="64" t="n"/>
       <c r="AA42" s="34" t="n"/>
       <c r="AB42" s="52" t="inlineStr"/>
-      <c r="AC42" s="34" t="n"/>
+      <c r="AC42" s="62" t="n"/>
       <c r="AD42" s="54" t="inlineStr"/>
       <c r="AE42" s="55" t="inlineStr"/>
     </row>
@@ -4170,13 +4185,13 @@
       <c r="T43" s="53" t="inlineStr"/>
       <c r="U43" s="53" t="inlineStr"/>
       <c r="V43" s="34" t="n"/>
-      <c r="W43" s="53" t="inlineStr"/>
-      <c r="X43" s="53" t="inlineStr"/>
-      <c r="Y43" s="53" t="inlineStr"/>
-      <c r="Z43" s="53" t="inlineStr"/>
+      <c r="W43" s="52" t="inlineStr"/>
+      <c r="X43" s="53" t="n"/>
+      <c r="Y43" s="53" t="n"/>
+      <c r="Z43" s="64" t="n"/>
       <c r="AA43" s="34" t="n"/>
       <c r="AB43" s="52" t="inlineStr"/>
-      <c r="AC43" s="34" t="n"/>
+      <c r="AC43" s="62" t="n"/>
       <c r="AD43" s="54" t="inlineStr"/>
       <c r="AE43" s="55" t="inlineStr"/>
     </row>
@@ -4211,13 +4226,13 @@
       <c r="T44" s="53" t="inlineStr"/>
       <c r="U44" s="53" t="inlineStr"/>
       <c r="V44" s="34" t="n"/>
-      <c r="W44" s="53" t="inlineStr"/>
-      <c r="X44" s="53" t="inlineStr"/>
-      <c r="Y44" s="53" t="inlineStr"/>
-      <c r="Z44" s="53" t="inlineStr"/>
+      <c r="W44" s="52" t="inlineStr"/>
+      <c r="X44" s="53" t="n"/>
+      <c r="Y44" s="53" t="n"/>
+      <c r="Z44" s="64" t="n"/>
       <c r="AA44" s="34" t="n"/>
       <c r="AB44" s="52" t="inlineStr"/>
-      <c r="AC44" s="34" t="n"/>
+      <c r="AC44" s="62" t="n"/>
       <c r="AD44" s="54" t="inlineStr"/>
       <c r="AE44" s="55" t="inlineStr"/>
     </row>
@@ -4252,13 +4267,13 @@
       <c r="T45" s="53" t="inlineStr"/>
       <c r="U45" s="53" t="inlineStr"/>
       <c r="V45" s="34" t="n"/>
-      <c r="W45" s="53" t="inlineStr"/>
-      <c r="X45" s="53" t="inlineStr"/>
-      <c r="Y45" s="53" t="inlineStr"/>
-      <c r="Z45" s="53" t="inlineStr"/>
+      <c r="W45" s="52" t="inlineStr"/>
+      <c r="X45" s="53" t="n"/>
+      <c r="Y45" s="53" t="n"/>
+      <c r="Z45" s="64" t="n"/>
       <c r="AA45" s="34" t="n"/>
       <c r="AB45" s="52" t="inlineStr"/>
-      <c r="AC45" s="34" t="n"/>
+      <c r="AC45" s="62" t="n"/>
       <c r="AD45" s="54" t="inlineStr"/>
       <c r="AE45" s="55" t="inlineStr"/>
     </row>
@@ -4293,13 +4308,13 @@
       <c r="T46" s="53" t="inlineStr"/>
       <c r="U46" s="53" t="inlineStr"/>
       <c r="V46" s="34" t="n"/>
-      <c r="W46" s="53" t="inlineStr"/>
-      <c r="X46" s="53" t="inlineStr"/>
-      <c r="Y46" s="53" t="inlineStr"/>
-      <c r="Z46" s="53" t="inlineStr"/>
+      <c r="W46" s="52" t="inlineStr"/>
+      <c r="X46" s="53" t="n"/>
+      <c r="Y46" s="53" t="n"/>
+      <c r="Z46" s="64" t="n"/>
       <c r="AA46" s="34" t="n"/>
       <c r="AB46" s="52" t="inlineStr"/>
-      <c r="AC46" s="34" t="n"/>
+      <c r="AC46" s="62" t="n"/>
       <c r="AD46" s="54" t="inlineStr"/>
       <c r="AE46" s="55" t="inlineStr"/>
     </row>
@@ -4334,13 +4349,13 @@
       <c r="T47" s="53" t="inlineStr"/>
       <c r="U47" s="53" t="inlineStr"/>
       <c r="V47" s="34" t="n"/>
-      <c r="W47" s="53" t="inlineStr"/>
-      <c r="X47" s="53" t="inlineStr"/>
-      <c r="Y47" s="53" t="inlineStr"/>
-      <c r="Z47" s="53" t="inlineStr"/>
+      <c r="W47" s="52" t="inlineStr"/>
+      <c r="X47" s="53" t="n"/>
+      <c r="Y47" s="53" t="n"/>
+      <c r="Z47" s="64" t="n"/>
       <c r="AA47" s="34" t="n"/>
       <c r="AB47" s="52" t="inlineStr"/>
-      <c r="AC47" s="34" t="n"/>
+      <c r="AC47" s="62" t="n"/>
       <c r="AD47" s="54" t="inlineStr"/>
       <c r="AE47" s="55" t="inlineStr"/>
     </row>
@@ -4375,13 +4390,13 @@
       <c r="T48" s="53" t="inlineStr"/>
       <c r="U48" s="53" t="inlineStr"/>
       <c r="V48" s="34" t="n"/>
-      <c r="W48" s="53" t="inlineStr"/>
-      <c r="X48" s="53" t="inlineStr"/>
-      <c r="Y48" s="53" t="inlineStr"/>
-      <c r="Z48" s="53" t="inlineStr"/>
+      <c r="W48" s="52" t="inlineStr"/>
+      <c r="X48" s="53" t="n"/>
+      <c r="Y48" s="53" t="n"/>
+      <c r="Z48" s="64" t="n"/>
       <c r="AA48" s="34" t="n"/>
       <c r="AB48" s="52" t="inlineStr"/>
-      <c r="AC48" s="34" t="n"/>
+      <c r="AC48" s="62" t="n"/>
       <c r="AD48" s="54" t="inlineStr"/>
       <c r="AE48" s="55" t="inlineStr"/>
     </row>
@@ -4416,13 +4431,13 @@
       <c r="T49" s="53" t="inlineStr"/>
       <c r="U49" s="53" t="inlineStr"/>
       <c r="V49" s="34" t="n"/>
-      <c r="W49" s="53" t="inlineStr"/>
-      <c r="X49" s="53" t="inlineStr"/>
-      <c r="Y49" s="53" t="inlineStr"/>
-      <c r="Z49" s="53" t="inlineStr"/>
+      <c r="W49" s="52" t="inlineStr"/>
+      <c r="X49" s="53" t="n"/>
+      <c r="Y49" s="53" t="n"/>
+      <c r="Z49" s="64" t="n"/>
       <c r="AA49" s="34" t="n"/>
       <c r="AB49" s="52" t="inlineStr"/>
-      <c r="AC49" s="34" t="n"/>
+      <c r="AC49" s="62" t="n"/>
       <c r="AD49" s="54" t="inlineStr"/>
       <c r="AE49" s="55" t="inlineStr"/>
     </row>
@@ -4457,13 +4472,13 @@
       <c r="T50" s="53" t="inlineStr"/>
       <c r="U50" s="53" t="inlineStr"/>
       <c r="V50" s="34" t="n"/>
-      <c r="W50" s="53" t="inlineStr"/>
-      <c r="X50" s="53" t="inlineStr"/>
-      <c r="Y50" s="53" t="inlineStr"/>
-      <c r="Z50" s="53" t="inlineStr"/>
+      <c r="W50" s="52" t="inlineStr"/>
+      <c r="X50" s="53" t="n"/>
+      <c r="Y50" s="53" t="n"/>
+      <c r="Z50" s="64" t="n"/>
       <c r="AA50" s="34" t="n"/>
       <c r="AB50" s="52" t="inlineStr"/>
-      <c r="AC50" s="34" t="n"/>
+      <c r="AC50" s="62" t="n"/>
       <c r="AD50" s="54" t="inlineStr"/>
       <c r="AE50" s="55" t="inlineStr"/>
     </row>
@@ -4498,13 +4513,13 @@
       <c r="T51" s="53" t="inlineStr"/>
       <c r="U51" s="53" t="inlineStr"/>
       <c r="V51" s="34" t="n"/>
-      <c r="W51" s="53" t="inlineStr"/>
-      <c r="X51" s="53" t="inlineStr"/>
-      <c r="Y51" s="53" t="inlineStr"/>
-      <c r="Z51" s="53" t="inlineStr"/>
+      <c r="W51" s="52" t="inlineStr"/>
+      <c r="X51" s="53" t="n"/>
+      <c r="Y51" s="53" t="n"/>
+      <c r="Z51" s="64" t="n"/>
       <c r="AA51" s="34" t="n"/>
       <c r="AB51" s="52" t="inlineStr"/>
-      <c r="AC51" s="34" t="n"/>
+      <c r="AC51" s="62" t="n"/>
       <c r="AD51" s="54" t="inlineStr"/>
       <c r="AE51" s="55" t="inlineStr"/>
     </row>
@@ -4539,13 +4554,13 @@
       <c r="T52" s="53" t="inlineStr"/>
       <c r="U52" s="53" t="inlineStr"/>
       <c r="V52" s="34" t="n"/>
-      <c r="W52" s="53" t="inlineStr"/>
-      <c r="X52" s="53" t="inlineStr"/>
-      <c r="Y52" s="53" t="inlineStr"/>
-      <c r="Z52" s="53" t="inlineStr"/>
+      <c r="W52" s="52" t="inlineStr"/>
+      <c r="X52" s="53" t="n"/>
+      <c r="Y52" s="53" t="n"/>
+      <c r="Z52" s="64" t="n"/>
       <c r="AA52" s="34" t="n"/>
       <c r="AB52" s="52" t="inlineStr"/>
-      <c r="AC52" s="34" t="n"/>
+      <c r="AC52" s="62" t="n"/>
       <c r="AD52" s="54" t="inlineStr"/>
       <c r="AE52" s="55" t="inlineStr"/>
     </row>
@@ -4580,13 +4595,13 @@
       <c r="T53" s="53" t="inlineStr"/>
       <c r="U53" s="53" t="inlineStr"/>
       <c r="V53" s="34" t="n"/>
-      <c r="W53" s="53" t="inlineStr"/>
-      <c r="X53" s="53" t="inlineStr"/>
-      <c r="Y53" s="53" t="inlineStr"/>
-      <c r="Z53" s="53" t="inlineStr"/>
+      <c r="W53" s="52" t="inlineStr"/>
+      <c r="X53" s="53" t="n"/>
+      <c r="Y53" s="53" t="n"/>
+      <c r="Z53" s="64" t="n"/>
       <c r="AA53" s="34" t="n"/>
       <c r="AB53" s="52" t="inlineStr"/>
-      <c r="AC53" s="34" t="n"/>
+      <c r="AC53" s="62" t="n"/>
       <c r="AD53" s="54" t="inlineStr"/>
       <c r="AE53" s="55" t="inlineStr"/>
     </row>
@@ -4621,13 +4636,13 @@
       <c r="T54" s="53" t="inlineStr"/>
       <c r="U54" s="53" t="inlineStr"/>
       <c r="V54" s="34" t="n"/>
-      <c r="W54" s="53" t="inlineStr"/>
-      <c r="X54" s="53" t="inlineStr"/>
-      <c r="Y54" s="53" t="inlineStr"/>
-      <c r="Z54" s="53" t="inlineStr"/>
+      <c r="W54" s="52" t="inlineStr"/>
+      <c r="X54" s="53" t="n"/>
+      <c r="Y54" s="53" t="n"/>
+      <c r="Z54" s="64" t="n"/>
       <c r="AA54" s="34" t="n"/>
       <c r="AB54" s="52" t="inlineStr"/>
-      <c r="AC54" s="34" t="n"/>
+      <c r="AC54" s="62" t="n"/>
       <c r="AD54" s="54" t="inlineStr"/>
       <c r="AE54" s="55" t="inlineStr"/>
     </row>
@@ -4662,13 +4677,13 @@
       <c r="T55" s="53" t="inlineStr"/>
       <c r="U55" s="53" t="inlineStr"/>
       <c r="V55" s="34" t="n"/>
-      <c r="W55" s="53" t="inlineStr"/>
-      <c r="X55" s="53" t="inlineStr"/>
-      <c r="Y55" s="53" t="inlineStr"/>
-      <c r="Z55" s="53" t="inlineStr"/>
+      <c r="W55" s="52" t="inlineStr"/>
+      <c r="X55" s="53" t="n"/>
+      <c r="Y55" s="53" t="n"/>
+      <c r="Z55" s="64" t="n"/>
       <c r="AA55" s="34" t="n"/>
       <c r="AB55" s="52" t="inlineStr"/>
-      <c r="AC55" s="34" t="n"/>
+      <c r="AC55" s="62" t="n"/>
       <c r="AD55" s="54" t="inlineStr"/>
       <c r="AE55" s="55" t="inlineStr"/>
     </row>
@@ -4703,13 +4718,13 @@
       <c r="T56" s="53" t="inlineStr"/>
       <c r="U56" s="53" t="inlineStr"/>
       <c r="V56" s="34" t="n"/>
-      <c r="W56" s="53" t="inlineStr"/>
-      <c r="X56" s="53" t="inlineStr"/>
-      <c r="Y56" s="53" t="inlineStr"/>
-      <c r="Z56" s="53" t="inlineStr"/>
+      <c r="W56" s="52" t="inlineStr"/>
+      <c r="X56" s="53" t="n"/>
+      <c r="Y56" s="53" t="n"/>
+      <c r="Z56" s="64" t="n"/>
       <c r="AA56" s="34" t="n"/>
       <c r="AB56" s="52" t="inlineStr"/>
-      <c r="AC56" s="34" t="n"/>
+      <c r="AC56" s="62" t="n"/>
       <c r="AD56" s="54" t="inlineStr"/>
       <c r="AE56" s="55" t="inlineStr"/>
     </row>
@@ -4744,13 +4759,13 @@
       <c r="T57" s="53" t="inlineStr"/>
       <c r="U57" s="53" t="inlineStr"/>
       <c r="V57" s="34" t="n"/>
-      <c r="W57" s="53" t="inlineStr"/>
-      <c r="X57" s="53" t="inlineStr"/>
-      <c r="Y57" s="53" t="inlineStr"/>
-      <c r="Z57" s="53" t="inlineStr"/>
+      <c r="W57" s="52" t="inlineStr"/>
+      <c r="X57" s="53" t="n"/>
+      <c r="Y57" s="53" t="n"/>
+      <c r="Z57" s="64" t="n"/>
       <c r="AA57" s="34" t="n"/>
       <c r="AB57" s="52" t="inlineStr"/>
-      <c r="AC57" s="34" t="n"/>
+      <c r="AC57" s="62" t="n"/>
       <c r="AD57" s="54" t="inlineStr"/>
       <c r="AE57" s="55" t="inlineStr"/>
     </row>
@@ -4785,13 +4800,13 @@
       <c r="T58" s="53" t="inlineStr"/>
       <c r="U58" s="53" t="inlineStr"/>
       <c r="V58" s="34" t="n"/>
-      <c r="W58" s="53" t="inlineStr"/>
-      <c r="X58" s="53" t="inlineStr"/>
-      <c r="Y58" s="53" t="inlineStr"/>
-      <c r="Z58" s="53" t="inlineStr"/>
+      <c r="W58" s="52" t="inlineStr"/>
+      <c r="X58" s="53" t="n"/>
+      <c r="Y58" s="53" t="n"/>
+      <c r="Z58" s="64" t="n"/>
       <c r="AA58" s="34" t="n"/>
       <c r="AB58" s="52" t="inlineStr"/>
-      <c r="AC58" s="34" t="n"/>
+      <c r="AC58" s="62" t="n"/>
       <c r="AD58" s="54" t="inlineStr"/>
       <c r="AE58" s="55" t="inlineStr"/>
     </row>
@@ -4826,13 +4841,13 @@
       <c r="T59" s="53" t="inlineStr"/>
       <c r="U59" s="53" t="inlineStr"/>
       <c r="V59" s="34" t="n"/>
-      <c r="W59" s="53" t="inlineStr"/>
-      <c r="X59" s="53" t="inlineStr"/>
-      <c r="Y59" s="53" t="inlineStr"/>
-      <c r="Z59" s="53" t="inlineStr"/>
+      <c r="W59" s="52" t="inlineStr"/>
+      <c r="X59" s="53" t="n"/>
+      <c r="Y59" s="53" t="n"/>
+      <c r="Z59" s="64" t="n"/>
       <c r="AA59" s="34" t="n"/>
       <c r="AB59" s="52" t="inlineStr"/>
-      <c r="AC59" s="34" t="n"/>
+      <c r="AC59" s="62" t="n"/>
       <c r="AD59" s="54" t="inlineStr"/>
       <c r="AE59" s="55" t="inlineStr"/>
     </row>
@@ -4867,13 +4882,13 @@
       <c r="T60" s="53" t="inlineStr"/>
       <c r="U60" s="53" t="inlineStr"/>
       <c r="V60" s="34" t="n"/>
-      <c r="W60" s="53" t="inlineStr"/>
-      <c r="X60" s="53" t="inlineStr"/>
-      <c r="Y60" s="53" t="inlineStr"/>
-      <c r="Z60" s="53" t="inlineStr"/>
+      <c r="W60" s="52" t="inlineStr"/>
+      <c r="X60" s="53" t="n"/>
+      <c r="Y60" s="53" t="n"/>
+      <c r="Z60" s="64" t="n"/>
       <c r="AA60" s="34" t="n"/>
       <c r="AB60" s="52" t="inlineStr"/>
-      <c r="AC60" s="34" t="n"/>
+      <c r="AC60" s="62" t="n"/>
       <c r="AD60" s="54" t="inlineStr"/>
       <c r="AE60" s="55" t="inlineStr"/>
     </row>
@@ -4908,13 +4923,13 @@
       <c r="T61" s="53" t="inlineStr"/>
       <c r="U61" s="53" t="inlineStr"/>
       <c r="V61" s="34" t="n"/>
-      <c r="W61" s="53" t="inlineStr"/>
-      <c r="X61" s="53" t="inlineStr"/>
-      <c r="Y61" s="53" t="inlineStr"/>
-      <c r="Z61" s="53" t="inlineStr"/>
+      <c r="W61" s="52" t="inlineStr"/>
+      <c r="X61" s="53" t="n"/>
+      <c r="Y61" s="53" t="n"/>
+      <c r="Z61" s="64" t="n"/>
       <c r="AA61" s="34" t="n"/>
       <c r="AB61" s="52" t="inlineStr"/>
-      <c r="AC61" s="34" t="n"/>
+      <c r="AC61" s="62" t="n"/>
       <c r="AD61" s="54" t="inlineStr"/>
       <c r="AE61" s="55" t="inlineStr"/>
     </row>
@@ -4949,13 +4964,13 @@
       <c r="T62" s="53" t="inlineStr"/>
       <c r="U62" s="53" t="inlineStr"/>
       <c r="V62" s="34" t="n"/>
-      <c r="W62" s="53" t="inlineStr"/>
-      <c r="X62" s="53" t="inlineStr"/>
-      <c r="Y62" s="53" t="inlineStr"/>
-      <c r="Z62" s="53" t="inlineStr"/>
+      <c r="W62" s="52" t="inlineStr"/>
+      <c r="X62" s="53" t="n"/>
+      <c r="Y62" s="53" t="n"/>
+      <c r="Z62" s="64" t="n"/>
       <c r="AA62" s="34" t="n"/>
       <c r="AB62" s="52" t="inlineStr"/>
-      <c r="AC62" s="34" t="n"/>
+      <c r="AC62" s="62" t="n"/>
       <c r="AD62" s="54" t="inlineStr"/>
       <c r="AE62" s="55" t="inlineStr"/>
     </row>
@@ -4990,13 +5005,13 @@
       <c r="T63" s="53" t="inlineStr"/>
       <c r="U63" s="53" t="inlineStr"/>
       <c r="V63" s="34" t="n"/>
-      <c r="W63" s="53" t="inlineStr"/>
-      <c r="X63" s="53" t="inlineStr"/>
-      <c r="Y63" s="53" t="inlineStr"/>
-      <c r="Z63" s="53" t="inlineStr"/>
+      <c r="W63" s="52" t="inlineStr"/>
+      <c r="X63" s="53" t="n"/>
+      <c r="Y63" s="53" t="n"/>
+      <c r="Z63" s="64" t="n"/>
       <c r="AA63" s="34" t="n"/>
       <c r="AB63" s="52" t="inlineStr"/>
-      <c r="AC63" s="34" t="n"/>
+      <c r="AC63" s="62" t="n"/>
       <c r="AD63" s="54" t="inlineStr"/>
       <c r="AE63" s="55" t="inlineStr"/>
     </row>
@@ -5031,13 +5046,13 @@
       <c r="T64" s="53" t="inlineStr"/>
       <c r="U64" s="53" t="inlineStr"/>
       <c r="V64" s="34" t="n"/>
-      <c r="W64" s="53" t="inlineStr"/>
-      <c r="X64" s="53" t="inlineStr"/>
-      <c r="Y64" s="53" t="inlineStr"/>
-      <c r="Z64" s="53" t="inlineStr"/>
+      <c r="W64" s="52" t="inlineStr"/>
+      <c r="X64" s="53" t="n"/>
+      <c r="Y64" s="53" t="n"/>
+      <c r="Z64" s="64" t="n"/>
       <c r="AA64" s="34" t="n"/>
       <c r="AB64" s="52" t="inlineStr"/>
-      <c r="AC64" s="34" t="n"/>
+      <c r="AC64" s="62" t="n"/>
       <c r="AD64" s="54" t="inlineStr"/>
       <c r="AE64" s="55" t="inlineStr"/>
     </row>
@@ -5072,13 +5087,13 @@
       <c r="T65" s="53" t="inlineStr"/>
       <c r="U65" s="53" t="inlineStr"/>
       <c r="V65" s="34" t="n"/>
-      <c r="W65" s="53" t="inlineStr"/>
-      <c r="X65" s="53" t="inlineStr"/>
-      <c r="Y65" s="53" t="inlineStr"/>
-      <c r="Z65" s="53" t="inlineStr"/>
+      <c r="W65" s="52" t="inlineStr"/>
+      <c r="X65" s="53" t="n"/>
+      <c r="Y65" s="53" t="n"/>
+      <c r="Z65" s="64" t="n"/>
       <c r="AA65" s="34" t="n"/>
       <c r="AB65" s="52" t="inlineStr"/>
-      <c r="AC65" s="34" t="n"/>
+      <c r="AC65" s="62" t="n"/>
       <c r="AD65" s="54" t="inlineStr"/>
       <c r="AE65" s="55" t="inlineStr"/>
     </row>
@@ -5113,13 +5128,13 @@
       <c r="T66" s="53" t="inlineStr"/>
       <c r="U66" s="53" t="inlineStr"/>
       <c r="V66" s="34" t="n"/>
-      <c r="W66" s="53" t="inlineStr"/>
-      <c r="X66" s="53" t="inlineStr"/>
-      <c r="Y66" s="53" t="inlineStr"/>
-      <c r="Z66" s="53" t="inlineStr"/>
+      <c r="W66" s="52" t="inlineStr"/>
+      <c r="X66" s="53" t="n"/>
+      <c r="Y66" s="53" t="n"/>
+      <c r="Z66" s="64" t="n"/>
       <c r="AA66" s="34" t="n"/>
       <c r="AB66" s="52" t="inlineStr"/>
-      <c r="AC66" s="34" t="n"/>
+      <c r="AC66" s="62" t="n"/>
       <c r="AD66" s="54" t="inlineStr"/>
       <c r="AE66" s="55" t="inlineStr"/>
     </row>
@@ -5154,13 +5169,13 @@
       <c r="T67" s="53" t="inlineStr"/>
       <c r="U67" s="53" t="inlineStr"/>
       <c r="V67" s="34" t="n"/>
-      <c r="W67" s="53" t="inlineStr"/>
-      <c r="X67" s="53" t="inlineStr"/>
-      <c r="Y67" s="53" t="inlineStr"/>
-      <c r="Z67" s="53" t="inlineStr"/>
+      <c r="W67" s="52" t="inlineStr"/>
+      <c r="X67" s="53" t="n"/>
+      <c r="Y67" s="53" t="n"/>
+      <c r="Z67" s="64" t="n"/>
       <c r="AA67" s="34" t="n"/>
       <c r="AB67" s="52" t="inlineStr"/>
-      <c r="AC67" s="34" t="n"/>
+      <c r="AC67" s="62" t="n"/>
       <c r="AD67" s="54" t="inlineStr"/>
       <c r="AE67" s="55" t="inlineStr"/>
     </row>
@@ -5195,13 +5210,13 @@
       <c r="T68" s="53" t="inlineStr"/>
       <c r="U68" s="53" t="inlineStr"/>
       <c r="V68" s="34" t="n"/>
-      <c r="W68" s="53" t="inlineStr"/>
-      <c r="X68" s="53" t="inlineStr"/>
-      <c r="Y68" s="53" t="inlineStr"/>
-      <c r="Z68" s="53" t="inlineStr"/>
+      <c r="W68" s="52" t="inlineStr"/>
+      <c r="X68" s="53" t="n"/>
+      <c r="Y68" s="53" t="n"/>
+      <c r="Z68" s="64" t="n"/>
       <c r="AA68" s="34" t="n"/>
       <c r="AB68" s="52" t="inlineStr"/>
-      <c r="AC68" s="34" t="n"/>
+      <c r="AC68" s="62" t="n"/>
       <c r="AD68" s="54" t="inlineStr"/>
       <c r="AE68" s="55" t="inlineStr"/>
     </row>
@@ -5210,13 +5225,13 @@
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="AE4:AE8"/>
     <mergeCell ref="AB4"/>
-    <mergeCell ref="W4:Z4"/>
     <mergeCell ref="D4:F4"/>
     <mergeCell ref="B4:B8"/>
     <mergeCell ref="H4:J4"/>
     <mergeCell ref="A1:AE1"/>
     <mergeCell ref="AD4:AD8"/>
     <mergeCell ref="A4:A8"/>
+    <mergeCell ref="W4:Y4"/>
     <mergeCell ref="J2:M2"/>
     <mergeCell ref="L4:N4"/>
     <mergeCell ref="C2:F2"/>

</xml_diff>

<commit_message>
Grille Excel : mettre à jour les phases 1 et 3 dans Instructions
- Phase 1 : renommer "Pilote (5 CR)", ajouter objectif test de l'outil
- Phase 3 : 75 CR total, chaque expert évalue 50 CR dont 25 communs, sans mention du modèle

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/grille_evaluation_CR.xlsx
+++ b/grille_evaluation_CR.xlsx
@@ -869,12 +869,12 @@
     <row r="7" ht="50" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Phase 1 — Pilote (membres du labo)</t>
+          <t>Phase 1 — Pilote (5 CR)</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Un premier test de la grille est réalisé en interne avec les membres de l'équipe de recherche sur un petit nombre de CR. L'objectif est de vérifier la clarté des critères, d'identifier les ambiguïtés et d'ajuster la grille si nécessaire avant de la soumettre aux experts cliniques.</t>
+          <t>Un premier test de la grille et de l'outil d'évaluation est réalisé en interne avec des membres de l'équipe de recherche sur 5 comptes rendus. L'objectif est double : vérifier la clarté des critères et identifier les ambiguïtés, mais aussi tester le bon fonctionnement de l'interface d'évaluation avant de la soumettre aux experts cliniques.</t>
         </is>
       </c>
     </row>
@@ -893,12 +893,12 @@
     <row r="9" ht="60" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Phase 3 — Évaluation finale (60 CR)</t>
+          <t>Phase 3 — Évaluation finale (75 CR)</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Chaque expert évalue 60 comptes rendus synthétiques (30 générés par Apertus-8B en 0-shot, 30 par Apertus-70B en 5-shot, température T=0,5). Un sous-ensemble de CR est évalué par les deux médecins radiothérapeutes simultanément (overlap, identifiés par * dans la grille) afin de surveiller la cohérence inter-annotateurs tout au long de l'évaluation.</t>
+          <t>Le corpus comprend 75 comptes rendus synthétiques. Chaque expert évalue 50 CR, dont 25 sont communs à plusieurs évaluateurs (overlap inter-annotateurs, identifiés par * dans la grille) afin de surveiller la cohérence inter-annotateurs tout au long de l'évaluation. Au total, l'ensemble des 75 CR sont couverts par au moins un évaluateur.</t>
         </is>
       </c>
     </row>
@@ -1078,7 +1078,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I31"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2128,8 +2128,6 @@
       </c>
       <c r="I29" s="25" t="n"/>
     </row>
-    <row r="30"/>
-    <row r="31"/>
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="A2:I2"/>

</xml_diff>